<commit_message>
fix: a regenerated one-cell or absolute anchor keeps the box Excel showed (#782)
A resized row inside a oneCell picture or above an absolute one makes the writer regenerate the anchor from the model; Excel keeps both at 96 x 57.6 pt, so the model's anchor-box size and position are written.

ImageAnchors.xlsx (drawing2, drawing3) and picture-webp.xlsx (drawing1) are regenerated: their twoCell pictures now write a:xfrm ext at the anchor box, the size Excel shows them at, instead of the stale size the file carried. Markers are unchanged.
</commit_message>
<xml_diff>
--- a/XLibur.Tests/Resource/Examples/ImageHandling/ImageAnchors.xlsx
+++ b/XLibur.Tests/Resource/Examples/ImageHandling/ImageAnchors.xlsx
@@ -171,7 +171,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="0" y="0"/>
-          <a:ext cx="2400300" cy="1447800"/>
+          <a:ext cx="1219200" cy="571500"/>
         </a:xfrm>
         <a:prstGeom prst="rect"/>
       </xdr:spPr>
@@ -212,7 +212,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="0" y="0"/>
-          <a:ext cx="3810000" cy="3810000"/>
+          <a:ext cx="1828800" cy="571500"/>
         </a:xfrm>
         <a:prstGeom prst="rect"/>
       </xdr:spPr>
@@ -248,7 +248,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="0" y="0"/>
-          <a:ext cx="3810000" cy="3810000"/>
+          <a:ext cx="1924050" cy="619125"/>
         </a:xfrm>
         <a:prstGeom prst="rect"/>
       </xdr:spPr>

</xml_diff>

<commit_message>
fix: a save writes a loaded picture back into its own anchor and keeps its styling (#843)
Every save rebuilt each picture's anchor with a bare spPr and blipFill, so rotation, borders,
shadows, crops and recolours Excel wrote were lost on the first save. A loaded picture is now
patched in place: only what changed (name, image link, position, size) is written. A sheet whose
pictures did not change is not touched, an image is fed only when it changed, and drawing ids are
no longer renumbered.
</commit_message>
<xml_diff>
--- a/XLibur.Tests/Resource/Examples/ImageHandling/ImageAnchors.xlsx
+++ b/XLibur.Tests/Resource/Examples/ImageHandling/ImageAnchors.xlsx
@@ -171,7 +171,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="0" y="0"/>
-          <a:ext cx="1219200" cy="571500"/>
+          <a:ext cx="2400300" cy="1447800"/>
         </a:xfrm>
         <a:prstGeom prst="rect"/>
       </xdr:spPr>
@@ -212,7 +212,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="0" y="0"/>
-          <a:ext cx="1828800" cy="571500"/>
+          <a:ext cx="3810000" cy="3810000"/>
         </a:xfrm>
         <a:prstGeom prst="rect"/>
       </xdr:spPr>
@@ -248,7 +248,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="0" y="0"/>
-          <a:ext cx="1924050" cy="619125"/>
+          <a:ext cx="3810000" cy="3810000"/>
         </a:xfrm>
         <a:prstGeom prst="rect"/>
       </xdr:spPr>

</xml_diff>